<commit_message>
Excel: corrige desfase en gráficos de Factores, orientación horizontal y PDF
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011cn2oC8KdNw1PNn42kUjFm
</commit_message>
<xml_diff>
--- a/analisis/resultados/Informe_morosidad.xlsx
+++ b/analisis/resultados/Informe_morosidad.xlsx
@@ -1005,11 +1005,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="23695412"/>
-        <c:axId val="36270690"/>
+        <c:axId val="24591755"/>
+        <c:axId val="51279698"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="23695412"/>
+        <c:axId val="24591755"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1041,7 +1041,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36270690"/>
+        <c:crossAx val="51279698"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1049,7 +1049,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36270690"/>
+        <c:axId val="51279698"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1115,7 +1115,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23695412"/>
+        <c:crossAx val="24591755"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1191,17 +1191,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Factores!E15</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>50.2%</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="1f5f8b"/>
@@ -1266,17 +1255,20 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Factores!$E$16:$E$18</c:f>
+              <c:f>Factores!$E$15:$E$18</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>0.502293577981651</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>0.415233415233415</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>0.533333333333333</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>0.272727272727273</c:v>
                 </c:pt>
               </c:numCache>
@@ -1285,11 +1277,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="81844308"/>
-        <c:axId val="69577230"/>
+        <c:axId val="30909741"/>
+        <c:axId val="71539176"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81844308"/>
+        <c:axId val="30909741"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1321,7 +1313,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69577230"/>
+        <c:crossAx val="71539176"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1329,7 +1321,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69577230"/>
+        <c:axId val="71539176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1395,7 +1387,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81844308"/>
+        <c:crossAx val="30909741"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1471,17 +1463,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Factores!E19</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>42.5%</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="1f5f8b"/>
@@ -1549,20 +1530,23 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Factores!$E$20:$E$23</c:f>
+              <c:f>Factores!$E$19:$E$23</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
+                  <c:v>0.425</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>0.47972972972973</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>0.450980392156863</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>0.403669724770642</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>0.568965517241379</c:v>
                 </c:pt>
               </c:numCache>
@@ -1571,11 +1555,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="98436567"/>
-        <c:axId val="48178873"/>
+        <c:axId val="34701450"/>
+        <c:axId val="77475185"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="98436567"/>
+        <c:axId val="34701450"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1607,7 +1591,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48178873"/>
+        <c:crossAx val="77475185"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1615,7 +1599,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48178873"/>
+        <c:axId val="77475185"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1681,7 +1665,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98436567"/>
+        <c:crossAx val="34701450"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1848,11 +1832,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1757397"/>
-        <c:axId val="21625428"/>
+        <c:axId val="76884899"/>
+        <c:axId val="61058276"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1757397"/>
+        <c:axId val="76884899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1884,7 +1868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21625428"/>
+        <c:crossAx val="61058276"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1892,7 +1876,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21625428"/>
+        <c:axId val="61058276"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1958,7 +1942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1757397"/>
+        <c:crossAx val="76884899"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2142,11 +2126,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52454440"/>
-        <c:axId val="2925296"/>
+        <c:axId val="76217730"/>
+        <c:axId val="23731570"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52454440"/>
+        <c:axId val="76217730"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2178,7 +2162,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2925296"/>
+        <c:crossAx val="23731570"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2186,7 +2170,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2925296"/>
+        <c:axId val="23731570"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2252,7 +2236,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52454440"/>
+        <c:crossAx val="76217730"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2412,11 +2396,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="48272437"/>
-        <c:axId val="46696170"/>
+        <c:axId val="91782586"/>
+        <c:axId val="20601405"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48272437"/>
+        <c:axId val="91782586"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2448,7 +2432,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46696170"/>
+        <c:crossAx val="20601405"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2456,7 +2440,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46696170"/>
+        <c:axId val="20601405"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2522,7 +2506,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48272437"/>
+        <c:crossAx val="91782586"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2700,11 +2684,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25018221"/>
-        <c:axId val="85294934"/>
+        <c:axId val="8124159"/>
+        <c:axId val="26040419"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25018221"/>
+        <c:axId val="8124159"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2736,7 +2720,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85294934"/>
+        <c:crossAx val="26040419"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2744,7 +2728,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85294934"/>
+        <c:axId val="26040419"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2810,7 +2794,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25018221"/>
+        <c:crossAx val="8124159"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2982,11 +2966,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="24718693"/>
-        <c:axId val="3585533"/>
+        <c:axId val="32592541"/>
+        <c:axId val="47637579"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24718693"/>
+        <c:axId val="32592541"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3018,7 +3002,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3585533"/>
+        <c:crossAx val="47637579"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3026,7 +3010,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3585533"/>
+        <c:axId val="47637579"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3092,7 +3076,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24718693"/>
+        <c:crossAx val="32592541"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3270,11 +3254,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="96330413"/>
-        <c:axId val="22529326"/>
+        <c:axId val="29639779"/>
+        <c:axId val="37031883"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="96330413"/>
+        <c:axId val="29639779"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3306,7 +3290,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22529326"/>
+        <c:crossAx val="37031883"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3314,7 +3298,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22529326"/>
+        <c:axId val="37031883"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3380,7 +3364,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96330413"/>
+        <c:crossAx val="29639779"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3558,11 +3542,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="69570640"/>
-        <c:axId val="79115111"/>
+        <c:axId val="94271999"/>
+        <c:axId val="10295195"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="69570640"/>
+        <c:axId val="94271999"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3594,7 +3578,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79115111"/>
+        <c:crossAx val="10295195"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3602,7 +3586,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79115111"/>
+        <c:axId val="10295195"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3668,7 +3652,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69570640"/>
+        <c:crossAx val="94271999"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3744,17 +3728,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Factores!E6</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>7.2%</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="1f5f8b"/>
@@ -3819,17 +3792,20 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Factores!$E$7:$E$9</c:f>
+              <c:f>Factores!$E$6:$E$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>0.0724946695095949</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>0.928039702233251</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>0.037037037037037</c:v>
                 </c:pt>
               </c:numCache>
@@ -3838,11 +3814,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="10648225"/>
-        <c:axId val="52318613"/>
+        <c:axId val="58905996"/>
+        <c:axId val="61347167"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10648225"/>
+        <c:axId val="58905996"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3874,7 +3850,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52318613"/>
+        <c:crossAx val="61347167"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3882,7 +3858,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52318613"/>
+        <c:axId val="61347167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3948,7 +3924,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10648225"/>
+        <c:crossAx val="58905996"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4024,17 +4000,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Factores!E11</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>41.5%</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="1f5f8b"/>
@@ -4099,17 +4064,20 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Factores!$E$12:$E$14</c:f>
+              <c:f>Factores!$E$11:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>0.414835164835165</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>0.558139534883721</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>0.605555555555556</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>0.27741935483871</c:v>
                 </c:pt>
               </c:numCache>
@@ -4118,11 +4086,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="4292005"/>
-        <c:axId val="94231495"/>
+        <c:axId val="1411455"/>
+        <c:axId val="75705888"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="4292005"/>
+        <c:axId val="1411455"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4154,7 +4122,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94231495"/>
+        <c:crossAx val="75705888"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4162,7 +4130,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94231495"/>
+        <c:axId val="75705888"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4228,7 +4196,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4292005"/>
+        <c:crossAx val="1411455"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4355,6 +4323,36 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>160920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>147600</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>2880</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="14621040" y="571680"/>
+        <a:ext cx="5039640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
@@ -4368,7 +4366,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvPr id="4" name="Chart 3"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -4377,7 +4375,37 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>160920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>147600</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>2880</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="14621040" y="4191120"/>
+        <a:ext cx="5039640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4398,71 +4426,11 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvPr id="6" name="Chart 5"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8505720" y="7810560"/>
-        <a:ext cx="5039640" cy="2699640"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>147600</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>2880</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame>
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="8505720" y="11430000"/>
-        <a:ext cx="5039640" cy="2699640"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>147600</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>2880</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame>
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="8505720" y="14668560"/>
         <a:ext cx="5039640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -4814,7 +4782,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -5008,7 +4976,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5019,7 +4987,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -5202,7 +5170,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5214,7 +5182,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:G62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -5815,7 +5783,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5827,7 +5795,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6378,7 +6346,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6390,7 +6358,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6649,7 +6617,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6660,7 +6628,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6761,7 +6729,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6773,7 +6741,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6937,7 +6905,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>